<commit_message>
Add axis titles to all dashboard charts
</commit_message>
<xml_diff>
--- a/claims_dashboard.xlsx
+++ b/claims_dashboard.xlsx
@@ -273,7 +273,23 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Quarter</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -284,6 +300,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -371,7 +388,23 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Claim Status</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -382,8 +415,24 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Claim Count</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -460,6 +509,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <title>
           <tx>
@@ -470,7 +520,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Month</a:t>
+                  <a:t>Report Month</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -486,6 +536,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <title>
@@ -573,7 +624,23 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Injury Cause</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -584,8 +651,24 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Claim Count</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -656,7 +739,23 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Injury Body Part</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -667,8 +766,24 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Total Incurred Loss ($)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -24077,7 +24192,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Claims Analytics — Executive KPIs</t>
+          <t>Claims Analytics - Executive KPIs</t>
         </is>
       </c>
     </row>
@@ -24269,7 +24384,7 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>NOTE: Slicers (School Level / Department / Status) require a live PivotTable connected to the "Data" sheet's ClaimsData table — see dashboard_pivot_slicer_guide.txt for exact steps.</t>
+          <t>NOTE: Slicers (School Level / Department / Status) require a live PivotTable connected to the "Data" sheet's ClaimsData table - see dashboard_pivot_slicer_guide.txt for exact steps.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix stale slicer note, sync README to v2 dashboard, tighten memo to one page
- claims_dashboard.xlsx: Pivot_Base was saved mid-filter (Elementary+Open
  only) in earlier versions, which looked like missing data - now saved
  showing the full unfiltered 375-claim dataset; replaced the stale
  "slicers require a live PivotTable" note (they now exist) with a note
  on the deliberate KPI-cards-vs-slicer-filtered-view split; slicers
  repositioned next to the KPI cards instead of sitting far below them
- README.md: describes the v2 dashboard (Pareto chart, pending-loss card,
  data-quality strip, live PivotTable/slicers) and adds
  build_live_dashboard.bas to the supplementary reference section
- findings_memo.pdf: tightened spacing so the exhibit chart fits on one
  page instead of spilling a paragraph onto a second page
</commit_message>
<xml_diff>
--- a/claims_dashboard.xlsx
+++ b/claims_dashboard.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/NikiChoksi/Documents/Niki/Projects/ClaimsAnalytics/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/NikiChoksi/Documents/Niki/Projects/ClaimsAnalytics/Claims_Analytics_Portfolio_NikiChoksi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C63D060D-FEC9-DF48-867F-D5F3352E8C85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D84DAA1D-3942-F543-8820-E83C8EE68D7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17540" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17540" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
   </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId6"/>
+    <pivotCache cacheId="2" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4632" uniqueCount="502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4640" uniqueCount="502">
   <si>
     <t>ClaimId</t>
   </si>
@@ -1498,7 +1498,7 @@
     <t>DATA QUALITY: 400 raw records -&gt; 15 exact duplicates removed -&gt; 3 missing IDs retained as UNASSIGNED-### -&gt; 10 exceptions quarantined -&gt; 375 clean records, of which 6 are pending a loss estimate (blank reserve, not zero). Full audit trail: claims_cleaning_log.xlsx.</t>
   </si>
   <si>
-    <t>NOTE: Slicers (School Level / Department / Status) require a live PivotTable connected to the "Data" sheet's ClaimsData table - see dashboard_pivot_slicer_guide.txt for exact steps.</t>
+    <t>KPI cards above reflect the full district (all 375 claims) as of the reporting period. The slicers below (School Level / Department / Status) filter the interactive Pivot_Base drill-down view, not the KPI cards - see dashboard_pivot_slicer_guide.txt for how they were built via build_live_dashboard.bas.</t>
   </si>
   <si>
     <t>Claims Trends</t>
@@ -1557,10 +1557,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="166" formatCode="[$-409]\$#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="[$-409]\$#,##0"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="165" formatCode="[$-409]\$#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="[$-409]\$#,##0"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -1575,58 +1575,68 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <color rgb="FF1F4E78"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF808080"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF595959"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="22"/>
       <color rgb="FF1F4E78"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="22"/>
       <color rgb="FF9C5700"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF375623"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9.5"/>
       <color rgb="FF1F4E78"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9.5"/>
       <color rgb="FF808080"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1676,13 +1686,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1691,10 +1701,14 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1702,11 +1716,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3300,7 +3309,7 @@
             <c:numRef>
               <c:f>Trends!$B$43:$B$53</c:f>
               <c:numCache>
-                <c:formatCode>\$#,##0</c:formatCode>
+                <c:formatCode>[$-409]\$#,##0</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
                   <c:v>275674.01</c:v>
@@ -3778,7 +3787,7 @@
             <c:numRef>
               <c:f>Trends!$B$99:$B$108</c:f>
               <c:numCache>
-                <c:formatCode>\$#,##0</c:formatCode>
+                <c:formatCode>[$-409]\$#,##0</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
                   <c:v>249306.76</c:v>
@@ -4432,19 +4441,19 @@
   </xdr:oneCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>84781</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>982869</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>173129</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>840946</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>88214</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>752597</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>10910</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="4" name="SchoolLevel">
@@ -4467,7 +4476,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -4477,8 +4486,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="0" y="8698694"/>
-              <a:ext cx="1912163" cy="1505346"/>
+              <a:off x="4637647" y="638796"/>
+              <a:ext cx="1914617" cy="1559336"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -4510,19 +4519,19 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>235106</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>38176</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>201976</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>159653</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>4126</xdr:colOff>
-      <xdr:row>44</xdr:row>
-      <xdr:rowOff>41609</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1042214</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>361869</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="5" name="Department">
@@ -4545,7 +4554,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -4555,8 +4564,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="2377541" y="8652089"/>
-              <a:ext cx="1911455" cy="1505346"/>
+              <a:off x="7074087" y="625320"/>
+              <a:ext cx="1912683" cy="1556882"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -4588,19 +4597,19 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>318743</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>166341</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>385003</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>688</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>87762</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>169774</xdr:rowOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>154021</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>26208</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="6" name="ClaimStatus">
@@ -4623,7 +4632,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -4633,8 +4642,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="4603613" y="8592515"/>
-              <a:ext cx="1911453" cy="1505346"/>
+              <a:off x="9402003" y="663910"/>
+              <a:ext cx="1913907" cy="1549520"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -4805,7 +4814,7 @@
     <cacheField name="ClaimId" numFmtId="0">
       <sharedItems/>
     </cacheField>
-    <cacheField name="ReportDate" numFmtId="165">
+    <cacheField name="ReportDate" numFmtId="164">
       <sharedItems containsSemiMixedTypes="0" containsNonDate="0" containsDate="1" containsString="0" minDate="2024-08-02T00:00:00" maxDate="2025-07-31T00:00:00"/>
     </cacheField>
     <cacheField name="SchoolSite" numFmtId="0">
@@ -4843,7 +4852,7 @@
         <s v="Re-opened"/>
       </sharedItems>
     </cacheField>
-    <cacheField name="IncurredLoss" numFmtId="166">
+    <cacheField name="IncurredLoss" numFmtId="165">
       <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="403.93" maxValue="21462"/>
     </cacheField>
     <cacheField name="LossIsEstimatePending" numFmtId="0">
@@ -10498,30 +10507,30 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{34E78ABF-4FC7-6E43-BF06-B3B80CA3B572}" name="PT_Master" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:E7" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{34E78ABF-4FC7-6E43-BF06-B3B80CA3B572}" name="PT_Master" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:I9" firstHeaderRow="1" firstDataRow="3" firstDataCol="1"/>
   <pivotFields count="13">
     <pivotField dataField="1" showAll="0"/>
-    <pivotField numFmtId="165" showAll="0"/>
+    <pivotField numFmtId="164" showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField axis="axisCol" showAll="0">
       <items count="4">
         <item x="1"/>
-        <item h="1" x="0"/>
-        <item h="1" x="2"/>
+        <item x="0"/>
+        <item x="2"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField showAll="0">
       <items count="9">
         <item x="7"/>
-        <item h="1" x="5"/>
-        <item h="1" x="6"/>
-        <item h="1" x="3"/>
-        <item h="1" x="4"/>
-        <item h="1" x="2"/>
-        <item h="1" x="1"/>
-        <item h="1" x="0"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item x="0"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -10529,9 +10538,9 @@
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
       <items count="4">
-        <item h="1" x="0"/>
+        <item x="0"/>
         <item x="1"/>
-        <item h="1" x="2"/>
+        <item x="2"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -10544,9 +10553,15 @@
   <rowFields count="1">
     <field x="7"/>
   </rowFields>
-  <rowItems count="2">
+  <rowItems count="4">
+    <i>
+      <x/>
+    </i>
     <i>
       <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
     </i>
     <i t="grand">
       <x/>
@@ -10556,9 +10571,23 @@
     <field x="3"/>
     <field x="-2"/>
   </colFields>
-  <colItems count="4">
+  <colItems count="8">
     <i>
       <x/>
+      <x/>
+    </i>
+    <i r="1" i="1">
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="1"/>
+      <x/>
+    </i>
+    <i r="1" i="1">
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
       <x/>
     </i>
     <i r="1" i="1">
@@ -10596,8 +10625,8 @@
     <tabular pivotCacheId="1084199705">
       <items count="3">
         <i x="1" s="1"/>
-        <i x="0"/>
-        <i x="2"/>
+        <i x="0" s="1"/>
+        <i x="2" s="1"/>
       </items>
     </tabular>
   </data>
@@ -10613,13 +10642,13 @@
     <tabular pivotCacheId="1084199705">
       <items count="8">
         <i x="7" s="1"/>
-        <i x="5"/>
-        <i x="6"/>
-        <i x="3"/>
-        <i x="4"/>
-        <i x="2"/>
-        <i x="1"/>
-        <i x="0"/>
+        <i x="5" s="1"/>
+        <i x="6" s="1"/>
+        <i x="3" s="1"/>
+        <i x="4" s="1"/>
+        <i x="2" s="1"/>
+        <i x="1" s="1"/>
+        <i x="0" s="1"/>
       </items>
     </tabular>
   </data>
@@ -10634,9 +10663,9 @@
   <data>
     <tabular pivotCacheId="1084199705">
       <items count="3">
-        <i x="0"/>
+        <i x="0" s="1"/>
         <i x="1" s="1"/>
-        <i x="2"/>
+        <i x="2" s="1"/>
       </items>
     </tabular>
   </data>
@@ -26324,7 +26353,10 @@
   <dimension ref="A1:M35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="13" width="14" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="2" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="13" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.25">
@@ -26341,56 +26373,52 @@
       <c r="A4" s="6" t="s">
         <v>460</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="D4" s="6" t="s">
+      <c r="B4" s="6" t="s">
         <v>461</v>
       </c>
+      <c r="C4" s="6" t="s">
+        <v>462</v>
+      </c>
       <c r="E4" s="7"/>
-      <c r="G4" s="6" t="s">
-        <v>462</v>
-      </c>
       <c r="H4" s="7"/>
     </row>
     <row r="5" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A5" s="8" t="s">
         <v>463</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="D5" s="8" t="s">
+      <c r="B5" s="8" t="s">
         <v>464</v>
       </c>
+      <c r="C5" s="8" t="s">
+        <v>465</v>
+      </c>
       <c r="E5" s="7"/>
-      <c r="G5" s="8" t="s">
-        <v>465</v>
-      </c>
       <c r="H5" s="7"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="6" t="s">
         <v>466</v>
       </c>
-      <c r="B8" s="7"/>
-      <c r="D8" s="6" t="s">
+      <c r="B8" s="6" t="s">
         <v>467</v>
       </c>
+      <c r="C8" s="6" t="s">
+        <v>468</v>
+      </c>
       <c r="E8" s="7"/>
-      <c r="G8" s="6" t="s">
-        <v>468</v>
-      </c>
       <c r="H8" s="7"/>
     </row>
     <row r="9" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="A9" s="8" t="s">
         <v>469</v>
       </c>
-      <c r="B9" s="7"/>
-      <c r="D9" s="8" t="s">
+      <c r="B9" s="8" t="s">
         <v>470</v>
       </c>
+      <c r="C9" s="8" t="s">
+        <v>471</v>
+      </c>
       <c r="E9" s="7"/>
-      <c r="G9" s="8" t="s">
-        <v>471</v>
-      </c>
       <c r="H9" s="7"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
@@ -26413,7 +26441,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="96" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:9" ht="80" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>476</v>
       </c>
@@ -26476,38 +26504,38 @@
       </c>
     </row>
     <row r="33" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="16" t="s">
+      <c r="A33" s="18" t="s">
         <v>483</v>
       </c>
-      <c r="B33" s="17"/>
-      <c r="C33" s="17"/>
-      <c r="D33" s="17"/>
-      <c r="E33" s="17"/>
-      <c r="F33" s="17"/>
-      <c r="G33" s="17"/>
-      <c r="H33" s="17"/>
-      <c r="I33" s="17"/>
-      <c r="J33" s="17"/>
-      <c r="K33" s="17"/>
-      <c r="L33" s="17"/>
-      <c r="M33" s="17"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="19"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="19"/>
+      <c r="F33" s="19"/>
+      <c r="G33" s="19"/>
+      <c r="H33" s="19"/>
+      <c r="I33" s="19"/>
+      <c r="J33" s="19"/>
+      <c r="K33" s="19"/>
+      <c r="L33" s="19"/>
+      <c r="M33" s="19"/>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A35" s="18" t="s">
+      <c r="A35" s="20" t="s">
         <v>484</v>
       </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="17"/>
-      <c r="G35" s="17"/>
-      <c r="H35" s="17"/>
-      <c r="I35" s="17"/>
-      <c r="J35" s="17"/>
-      <c r="K35" s="17"/>
-      <c r="L35" s="17"/>
-      <c r="M35" s="17"/>
+      <c r="B35" s="19"/>
+      <c r="C35" s="19"/>
+      <c r="D35" s="19"/>
+      <c r="E35" s="19"/>
+      <c r="F35" s="19"/>
+      <c r="G35" s="19"/>
+      <c r="H35" s="19"/>
+      <c r="I35" s="19"/>
+      <c r="J35" s="19"/>
+      <c r="K35" s="19"/>
+      <c r="L35" s="19"/>
+      <c r="M35" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -32492,38 +32520,44 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F2C47C2-71B1-7341-9B73-259726F816DE}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A3:E7"/>
+  <dimension ref="A3:I9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="18.1640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B3" s="19" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B3" s="16" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>24</v>
       </c>
       <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" t="s">
+        <v>95</v>
+      </c>
+      <c r="H4" t="s">
         <v>499</v>
       </c>
-      <c r="E4" t="s">
+      <c r="I4" t="s">
         <v>500</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A5" s="16" t="s">
         <v>495</v>
       </c>
       <c r="B5" t="s">
@@ -32532,39 +32566,133 @@
       <c r="C5" t="s">
         <v>501</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="20" t="s">
+      <c r="D5" t="s">
+        <v>498</v>
+      </c>
+      <c r="E5" t="s">
+        <v>501</v>
+      </c>
+      <c r="F5" t="s">
+        <v>498</v>
+      </c>
+      <c r="G5" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A6" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6">
+        <v>98</v>
+      </c>
+      <c r="C6">
+        <v>456914.27</v>
+      </c>
+      <c r="D6">
+        <v>60</v>
+      </c>
+      <c r="E6">
+        <v>185813.51</v>
+      </c>
+      <c r="F6">
+        <v>34</v>
+      </c>
+      <c r="G6">
+        <v>113024.66</v>
+      </c>
+      <c r="H6">
+        <v>192</v>
+      </c>
+      <c r="I6">
+        <v>755752.44000000029</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="21">
-        <v>11</v>
-      </c>
-      <c r="C6" s="21">
-        <v>56016.41</v>
-      </c>
-      <c r="D6" s="21">
-        <v>11</v>
-      </c>
-      <c r="E6" s="21">
-        <v>56016.41</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="20" t="s">
+      <c r="B7">
+        <v>74</v>
+      </c>
+      <c r="C7">
+        <v>315265.71000000002</v>
+      </c>
+      <c r="D7">
+        <v>41</v>
+      </c>
+      <c r="E7">
+        <v>182075.99000000002</v>
+      </c>
+      <c r="F7">
+        <v>25</v>
+      </c>
+      <c r="G7">
+        <v>90319.88</v>
+      </c>
+      <c r="H7">
+        <v>140</v>
+      </c>
+      <c r="I7">
+        <v>587661.57999999973</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8">
+        <v>20</v>
+      </c>
+      <c r="C8">
+        <v>66102.430000000008</v>
+      </c>
+      <c r="D8">
+        <v>17</v>
+      </c>
+      <c r="E8">
+        <v>79389.03</v>
+      </c>
+      <c r="F8">
+        <v>6</v>
+      </c>
+      <c r="G8">
+        <v>27976.459999999995</v>
+      </c>
+      <c r="H8">
+        <v>43</v>
+      </c>
+      <c r="I8">
+        <v>173467.91999999995</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9" s="17" t="s">
         <v>496</v>
       </c>
-      <c r="B7" s="21">
-        <v>11</v>
-      </c>
-      <c r="C7" s="21">
-        <v>56016.41</v>
-      </c>
-      <c r="D7" s="21">
-        <v>11</v>
-      </c>
-      <c r="E7" s="21">
-        <v>56016.41</v>
+      <c r="B9">
+        <v>192</v>
+      </c>
+      <c r="C9">
+        <v>838282.40999999992</v>
+      </c>
+      <c r="D9">
+        <v>118</v>
+      </c>
+      <c r="E9">
+        <v>447278.53</v>
+      </c>
+      <c r="F9">
+        <v>65</v>
+      </c>
+      <c r="G9">
+        <v>231321.00000000006</v>
+      </c>
+      <c r="H9">
+        <v>375</v>
+      </c>
+      <c r="I9">
+        <v>1516881.94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>